<commit_message>
Correct nine points in Point vs. Interval Estimation
The home-sales file is realistic teaching data, and its prices are roughly symmetric (skewness 0.06, which the notebook now prints), so the mean and median nearly agree. The interval is stated as 95% confidence in the procedure, the sample mean is efficient only for normal data, and comparing models needs an interval on the difference. The coverage figure draws 20 intervals with one miss, the standard-error bar spans the drawn bell, the part before this one has nine chapters, and the notebooks say 96 of 100 and sigma/sqrt(n).
</commit_message>
<xml_diff>
--- a/data/point-vs-interval-estimation--home_sales.xlsx
+++ b/data/point-vs-interval-estimation--home_sales.xlsx
@@ -8455,7 +8455,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WHAT IS CAPTURED: closed home-sale records, the kind a county assessor or MLS export produces.</t>
+          <t>WHAT IS CAPTURED: closed home-sale records, the kind a county assessor or MLS export produces (a realistic teaching dataset written for the book).</t>
         </is>
       </c>
     </row>
@@ -8469,7 +8469,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sale_price is right-skewed, so also compare the mean to the median.</t>
+          <t>Compare the mean to the median: these prices are roughly symmetric, though sale prices in many markets are right-skewed.</t>
         </is>
       </c>
     </row>

</xml_diff>